<commit_message>
fix: configure correct basename and base URL path for production deployment on GitHub Pages
</commit_message>
<xml_diff>
--- a/testing/selenium/selenium_report.xlsx
+++ b/testing/selenium/selenium_report.xlsx
@@ -3934,7 +3934,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="6">
-        <v>25</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3960,7 +3960,7 @@
         <v>14</v>
       </c>
       <c r="H3" s="8">
-        <v>36</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3986,7 +3986,7 @@
         <v>14</v>
       </c>
       <c r="H4" s="6">
-        <v>513</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4012,7 +4012,7 @@
         <v>14</v>
       </c>
       <c r="H5" s="8">
-        <v>89</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4038,7 +4038,7 @@
         <v>14</v>
       </c>
       <c r="H6" s="6">
-        <v>245</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4064,7 +4064,7 @@
         <v>14</v>
       </c>
       <c r="H7" s="8">
-        <v>62</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4090,7 +4090,7 @@
         <v>14</v>
       </c>
       <c r="H8" s="6">
-        <v>113</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4116,7 +4116,7 @@
         <v>14</v>
       </c>
       <c r="H9" s="8">
-        <v>137</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4142,7 +4142,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="6">
-        <v>159</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4168,7 +4168,7 @@
         <v>14</v>
       </c>
       <c r="H11" s="8">
-        <v>424</v>
+        <v>355</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4194,7 +4194,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="6">
-        <v>144</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4220,7 +4220,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="8">
-        <v>114</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4246,7 +4246,7 @@
         <v>14</v>
       </c>
       <c r="H14" s="6">
-        <v>125</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4272,7 +4272,7 @@
         <v>14</v>
       </c>
       <c r="H15" s="8">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4298,7 +4298,7 @@
         <v>14</v>
       </c>
       <c r="H16" s="6">
-        <v>196</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4324,7 +4324,7 @@
         <v>14</v>
       </c>
       <c r="H17" s="8">
-        <v>61</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4350,7 +4350,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="6">
-        <v>175</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4402,7 +4402,7 @@
         <v>14</v>
       </c>
       <c r="H20" s="6">
-        <v>66</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4428,7 +4428,7 @@
         <v>14</v>
       </c>
       <c r="H21" s="8">
-        <v>147</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4454,7 +4454,7 @@
         <v>14</v>
       </c>
       <c r="H22" s="6">
-        <v>133</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4480,7 +4480,7 @@
         <v>14</v>
       </c>
       <c r="H23" s="8">
-        <v>31</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4506,7 +4506,7 @@
         <v>14</v>
       </c>
       <c r="H24" s="6">
-        <v>119</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4532,7 +4532,7 @@
         <v>14</v>
       </c>
       <c r="H25" s="8">
-        <v>59</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4558,7 +4558,7 @@
         <v>14</v>
       </c>
       <c r="H26" s="6">
-        <v>116</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>14</v>
       </c>
       <c r="H27" s="8">
-        <v>46</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4610,7 +4610,7 @@
         <v>14</v>
       </c>
       <c r="H28" s="6">
-        <v>93</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4636,7 +4636,7 @@
         <v>14</v>
       </c>
       <c r="H29" s="8">
-        <v>565</v>
+        <v>441</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4662,7 +4662,7 @@
         <v>14</v>
       </c>
       <c r="H30" s="6">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4688,7 +4688,7 @@
         <v>14</v>
       </c>
       <c r="H31" s="8">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4714,7 +4714,7 @@
         <v>14</v>
       </c>
       <c r="H32" s="6">
-        <v>35</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4740,7 +4740,7 @@
         <v>14</v>
       </c>
       <c r="H33" s="8">
-        <v>148</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4766,7 +4766,7 @@
         <v>14</v>
       </c>
       <c r="H34" s="6">
-        <v>60</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4792,7 +4792,7 @@
         <v>14</v>
       </c>
       <c r="H35" s="8">
-        <v>133</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4818,7 +4818,7 @@
         <v>14</v>
       </c>
       <c r="H36" s="6">
-        <v>117</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4844,7 +4844,7 @@
         <v>14</v>
       </c>
       <c r="H37" s="8">
-        <v>59</v>
+        <v>162</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4870,7 +4870,7 @@
         <v>14</v>
       </c>
       <c r="H38" s="6">
-        <v>118</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4896,7 +4896,7 @@
         <v>14</v>
       </c>
       <c r="H39" s="8">
-        <v>197</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4922,7 +4922,7 @@
         <v>14</v>
       </c>
       <c r="H40" s="6">
-        <v>123</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4948,7 +4948,7 @@
         <v>14</v>
       </c>
       <c r="H41" s="8">
-        <v>67</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4974,7 +4974,7 @@
         <v>14</v>
       </c>
       <c r="H42" s="6">
-        <v>32</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5000,7 +5000,7 @@
         <v>14</v>
       </c>
       <c r="H43" s="8">
-        <v>187</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5026,7 +5026,7 @@
         <v>14</v>
       </c>
       <c r="H44" s="6">
-        <v>42</v>
+        <v>167</v>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5052,7 +5052,7 @@
         <v>14</v>
       </c>
       <c r="H45" s="8">
-        <v>31</v>
+        <v>82</v>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5078,7 +5078,7 @@
         <v>14</v>
       </c>
       <c r="H46" s="6">
-        <v>117</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5104,7 +5104,7 @@
         <v>14</v>
       </c>
       <c r="H47" s="8">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5130,7 +5130,7 @@
         <v>14</v>
       </c>
       <c r="H48" s="6">
-        <v>174</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5156,7 +5156,7 @@
         <v>14</v>
       </c>
       <c r="H49" s="8">
-        <v>186</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5182,7 +5182,7 @@
         <v>14</v>
       </c>
       <c r="H50" s="6">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5208,7 +5208,7 @@
         <v>14</v>
       </c>
       <c r="H51" s="8">
-        <v>108</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5234,7 +5234,7 @@
         <v>14</v>
       </c>
       <c r="H52" s="6">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5260,7 +5260,7 @@
         <v>14</v>
       </c>
       <c r="H53" s="8">
-        <v>66</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5286,7 +5286,7 @@
         <v>14</v>
       </c>
       <c r="H54" s="6">
-        <v>249</v>
+        <v>317</v>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5312,7 +5312,7 @@
         <v>14</v>
       </c>
       <c r="H55" s="8">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>14</v>
       </c>
       <c r="H56" s="6">
-        <v>123</v>
+        <v>134</v>
       </c>
     </row>
     <row r="57" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5364,7 +5364,7 @@
         <v>14</v>
       </c>
       <c r="H57" s="8">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5390,7 +5390,7 @@
         <v>14</v>
       </c>
       <c r="H58" s="6">
-        <v>142</v>
+        <v>127</v>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5416,7 +5416,7 @@
         <v>14</v>
       </c>
       <c r="H59" s="8">
-        <v>116</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5442,7 +5442,7 @@
         <v>14</v>
       </c>
       <c r="H60" s="6">
-        <v>156</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5468,7 +5468,7 @@
         <v>14</v>
       </c>
       <c r="H61" s="8">
-        <v>215</v>
+        <v>111</v>
       </c>
     </row>
     <row r="62" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5494,7 +5494,7 @@
         <v>14</v>
       </c>
       <c r="H62" s="6">
-        <v>194</v>
+        <v>57</v>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5520,7 +5520,7 @@
         <v>14</v>
       </c>
       <c r="H63" s="8">
-        <v>109</v>
+        <v>35</v>
       </c>
     </row>
     <row r="64" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5546,7 +5546,7 @@
         <v>14</v>
       </c>
       <c r="H64" s="6">
-        <v>135</v>
+        <v>70</v>
       </c>
     </row>
     <row r="65" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5572,7 +5572,7 @@
         <v>14</v>
       </c>
       <c r="H65" s="8">
-        <v>40</v>
+        <v>141</v>
       </c>
     </row>
     <row r="66" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5598,7 +5598,7 @@
         <v>14</v>
       </c>
       <c r="H66" s="6">
-        <v>159</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5624,7 +5624,7 @@
         <v>14</v>
       </c>
       <c r="H67" s="8">
-        <v>93</v>
+        <v>161</v>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5650,7 +5650,7 @@
         <v>14</v>
       </c>
       <c r="H68" s="6">
-        <v>155</v>
+        <v>196</v>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5676,7 +5676,7 @@
         <v>14</v>
       </c>
       <c r="H69" s="8">
-        <v>47</v>
+        <v>70</v>
       </c>
     </row>
     <row r="70" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5702,7 +5702,7 @@
         <v>14</v>
       </c>
       <c r="H70" s="6">
-        <v>103</v>
+        <v>169</v>
       </c>
     </row>
     <row r="71" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5728,7 +5728,7 @@
         <v>14</v>
       </c>
       <c r="H71" s="8">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5754,7 +5754,7 @@
         <v>14</v>
       </c>
       <c r="H72" s="6">
-        <v>190</v>
+        <v>122</v>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5780,7 +5780,7 @@
         <v>14</v>
       </c>
       <c r="H73" s="8">
-        <v>137</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5806,7 +5806,7 @@
         <v>14</v>
       </c>
       <c r="H74" s="6">
-        <v>204</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5832,7 +5832,7 @@
         <v>14</v>
       </c>
       <c r="H75" s="8">
-        <v>132</v>
+        <v>157</v>
       </c>
     </row>
     <row r="76" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5858,7 +5858,7 @@
         <v>14</v>
       </c>
       <c r="H76" s="6">
-        <v>91</v>
+        <v>56</v>
       </c>
     </row>
     <row r="77" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5884,7 +5884,7 @@
         <v>14</v>
       </c>
       <c r="H77" s="8">
-        <v>49</v>
+        <v>23</v>
       </c>
     </row>
     <row r="78" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5910,7 +5910,7 @@
         <v>14</v>
       </c>
       <c r="H78" s="6">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="79" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5936,7 +5936,7 @@
         <v>14</v>
       </c>
       <c r="H79" s="8">
-        <v>372</v>
+        <v>346</v>
       </c>
     </row>
     <row r="80" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5962,7 +5962,7 @@
         <v>14</v>
       </c>
       <c r="H80" s="6">
-        <v>49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -5988,7 +5988,7 @@
         <v>14</v>
       </c>
       <c r="H81" s="8">
-        <v>264</v>
+        <v>216</v>
       </c>
     </row>
     <row r="82" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6014,7 +6014,7 @@
         <v>14</v>
       </c>
       <c r="H82" s="6">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="83" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6040,7 +6040,7 @@
         <v>14</v>
       </c>
       <c r="H83" s="8">
-        <v>164</v>
+        <v>97</v>
       </c>
     </row>
     <row r="84" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6066,7 +6066,7 @@
         <v>14</v>
       </c>
       <c r="H84" s="6">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>14</v>
       </c>
       <c r="H85" s="8">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="86" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6118,7 +6118,7 @@
         <v>14</v>
       </c>
       <c r="H86" s="6">
-        <v>265</v>
+        <v>291</v>
       </c>
     </row>
     <row r="87" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6144,7 +6144,7 @@
         <v>14</v>
       </c>
       <c r="H87" s="8">
-        <v>189</v>
+        <v>149</v>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6170,7 +6170,7 @@
         <v>14</v>
       </c>
       <c r="H88" s="6">
-        <v>30</v>
+        <v>187</v>
       </c>
     </row>
     <row r="89" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6196,7 +6196,7 @@
         <v>14</v>
       </c>
       <c r="H89" s="8">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6222,7 +6222,7 @@
         <v>14</v>
       </c>
       <c r="H90" s="6">
-        <v>88</v>
+        <v>131</v>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6248,7 +6248,7 @@
         <v>14</v>
       </c>
       <c r="H91" s="8">
-        <v>87</v>
+        <v>173</v>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6274,7 +6274,7 @@
         <v>14</v>
       </c>
       <c r="H92" s="6">
-        <v>94</v>
+        <v>39</v>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6300,7 +6300,7 @@
         <v>14</v>
       </c>
       <c r="H93" s="8">
-        <v>112</v>
+        <v>167</v>
       </c>
     </row>
     <row r="94" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6326,7 +6326,7 @@
         <v>14</v>
       </c>
       <c r="H94" s="6">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6352,7 +6352,7 @@
         <v>14</v>
       </c>
       <c r="H95" s="8">
-        <v>111</v>
+        <v>76</v>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6378,7 +6378,7 @@
         <v>14</v>
       </c>
       <c r="H96" s="6">
-        <v>157</v>
+        <v>44</v>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6404,7 +6404,7 @@
         <v>14</v>
       </c>
       <c r="H97" s="8">
-        <v>108</v>
+        <v>182</v>
       </c>
     </row>
     <row r="98" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6430,7 +6430,7 @@
         <v>14</v>
       </c>
       <c r="H98" s="6">
-        <v>197</v>
+        <v>149</v>
       </c>
     </row>
     <row r="99" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6456,7 +6456,7 @@
         <v>14</v>
       </c>
       <c r="H99" s="8">
-        <v>33</v>
+        <v>57</v>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6482,7 +6482,7 @@
         <v>14</v>
       </c>
       <c r="H100" s="6">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6508,7 +6508,7 @@
         <v>14</v>
       </c>
       <c r="H101" s="8">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6534,7 +6534,7 @@
         <v>14</v>
       </c>
       <c r="H102" s="6">
-        <v>15</v>
+        <v>52</v>
       </c>
     </row>
     <row r="103" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6560,7 +6560,7 @@
         <v>14</v>
       </c>
       <c r="H103" s="8">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6586,7 +6586,7 @@
         <v>14</v>
       </c>
       <c r="H104" s="6">
-        <v>184</v>
+        <v>274</v>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6612,7 +6612,7 @@
         <v>14</v>
       </c>
       <c r="H105" s="8">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="106" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6638,7 +6638,7 @@
         <v>14</v>
       </c>
       <c r="H106" s="6">
-        <v>158</v>
+        <v>263</v>
       </c>
     </row>
     <row r="107" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6664,7 +6664,7 @@
         <v>14</v>
       </c>
       <c r="H107" s="8">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="108" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6690,7 +6690,7 @@
         <v>14</v>
       </c>
       <c r="H108" s="6">
-        <v>77</v>
+        <v>170</v>
       </c>
     </row>
     <row r="109" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6716,7 +6716,7 @@
         <v>14</v>
       </c>
       <c r="H109" s="8">
-        <v>87</v>
+        <v>146</v>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6742,7 +6742,7 @@
         <v>14</v>
       </c>
       <c r="H110" s="6">
-        <v>109</v>
+        <v>47</v>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6768,7 +6768,7 @@
         <v>14</v>
       </c>
       <c r="H111" s="8">
-        <v>433</v>
+        <v>253</v>
       </c>
     </row>
     <row r="112" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6794,7 +6794,7 @@
         <v>14</v>
       </c>
       <c r="H112" s="6">
-        <v>70</v>
+        <v>38</v>
       </c>
     </row>
     <row r="113" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6820,7 +6820,7 @@
         <v>14</v>
       </c>
       <c r="H113" s="8">
-        <v>96</v>
+        <v>161</v>
       </c>
     </row>
     <row r="114" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>14</v>
       </c>
       <c r="H114" s="6">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="115" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6872,7 +6872,7 @@
         <v>14</v>
       </c>
       <c r="H115" s="8">
-        <v>209</v>
+        <v>136</v>
       </c>
     </row>
     <row r="116" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6898,7 +6898,7 @@
         <v>14</v>
       </c>
       <c r="H116" s="6">
-        <v>110</v>
+        <v>176</v>
       </c>
     </row>
     <row r="117" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6924,7 +6924,7 @@
         <v>14</v>
       </c>
       <c r="H117" s="8">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="118" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6950,7 +6950,7 @@
         <v>14</v>
       </c>
       <c r="H118" s="6">
-        <v>148</v>
+        <v>94</v>
       </c>
     </row>
     <row r="119" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6976,7 +6976,7 @@
         <v>14</v>
       </c>
       <c r="H119" s="8">
-        <v>96</v>
+        <v>49</v>
       </c>
     </row>
     <row r="120" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7002,7 +7002,7 @@
         <v>14</v>
       </c>
       <c r="H120" s="6">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="121" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7028,7 +7028,7 @@
         <v>14</v>
       </c>
       <c r="H121" s="8">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="122" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7054,7 +7054,7 @@
         <v>14</v>
       </c>
       <c r="H122" s="6">
-        <v>112</v>
+        <v>198</v>
       </c>
     </row>
     <row r="123" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7080,7 +7080,7 @@
         <v>14</v>
       </c>
       <c r="H123" s="8">
-        <v>201</v>
+        <v>181</v>
       </c>
     </row>
     <row r="124" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7106,7 +7106,7 @@
         <v>14</v>
       </c>
       <c r="H124" s="6">
-        <v>137</v>
+        <v>186</v>
       </c>
     </row>
     <row r="125" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7132,7 +7132,7 @@
         <v>14</v>
       </c>
       <c r="H125" s="8">
-        <v>163</v>
+        <v>52</v>
       </c>
     </row>
     <row r="126" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7158,7 +7158,7 @@
         <v>14</v>
       </c>
       <c r="H126" s="6">
-        <v>122</v>
+        <v>65</v>
       </c>
     </row>
     <row r="127" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7184,7 +7184,7 @@
         <v>14</v>
       </c>
       <c r="H127" s="8">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7210,7 +7210,7 @@
         <v>14</v>
       </c>
       <c r="H128" s="6">
-        <v>84</v>
+        <v>61</v>
       </c>
     </row>
     <row r="129" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7236,7 +7236,7 @@
         <v>14</v>
       </c>
       <c r="H129" s="8">
-        <v>194</v>
+        <v>559</v>
       </c>
     </row>
     <row r="130" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7262,7 +7262,7 @@
         <v>14</v>
       </c>
       <c r="H130" s="6">
-        <v>46</v>
+        <v>55</v>
       </c>
     </row>
     <row r="131" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7288,7 +7288,7 @@
         <v>14</v>
       </c>
       <c r="H131" s="8">
-        <v>194</v>
+        <v>124</v>
       </c>
     </row>
     <row r="132" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7314,7 +7314,7 @@
         <v>14</v>
       </c>
       <c r="H132" s="6">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7340,7 +7340,7 @@
         <v>14</v>
       </c>
       <c r="H133" s="8">
-        <v>101</v>
+        <v>50</v>
       </c>
     </row>
     <row r="134" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7366,7 +7366,7 @@
         <v>14</v>
       </c>
       <c r="H134" s="6">
-        <v>147</v>
+        <v>51</v>
       </c>
     </row>
     <row r="135" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7418,7 +7418,7 @@
         <v>14</v>
       </c>
       <c r="H136" s="6">
-        <v>100</v>
+        <v>294</v>
       </c>
     </row>
     <row r="137" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7444,7 +7444,7 @@
         <v>14</v>
       </c>
       <c r="H137" s="8">
-        <v>140</v>
+        <v>131</v>
       </c>
     </row>
     <row r="138" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7470,7 +7470,7 @@
         <v>14</v>
       </c>
       <c r="H138" s="6">
-        <v>195</v>
+        <v>63</v>
       </c>
     </row>
     <row r="139" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7496,7 +7496,7 @@
         <v>14</v>
       </c>
       <c r="H139" s="8">
-        <v>103</v>
+        <v>177</v>
       </c>
     </row>
     <row r="140" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7522,7 +7522,7 @@
         <v>14</v>
       </c>
       <c r="H140" s="6">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="141" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7548,7 +7548,7 @@
         <v>14</v>
       </c>
       <c r="H141" s="8">
-        <v>50</v>
+        <v>148</v>
       </c>
     </row>
     <row r="142" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7574,7 +7574,7 @@
         <v>14</v>
       </c>
       <c r="H142" s="6">
-        <v>63</v>
+        <v>196</v>
       </c>
     </row>
     <row r="143" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>14</v>
       </c>
       <c r="H143" s="8">
-        <v>142</v>
+        <v>67</v>
       </c>
     </row>
     <row r="144" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7626,7 +7626,7 @@
         <v>14</v>
       </c>
       <c r="H144" s="6">
-        <v>74</v>
+        <v>92</v>
       </c>
     </row>
     <row r="145" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7652,7 +7652,7 @@
         <v>14</v>
       </c>
       <c r="H145" s="8">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="146" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7678,7 +7678,7 @@
         <v>14</v>
       </c>
       <c r="H146" s="6">
-        <v>128</v>
+        <v>57</v>
       </c>
     </row>
     <row r="147" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7704,7 +7704,7 @@
         <v>14</v>
       </c>
       <c r="H147" s="8">
-        <v>76</v>
+        <v>33</v>
       </c>
     </row>
     <row r="148" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7730,7 +7730,7 @@
         <v>14</v>
       </c>
       <c r="H148" s="6">
-        <v>157</v>
+        <v>88</v>
       </c>
     </row>
     <row r="149" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7756,7 +7756,7 @@
         <v>14</v>
       </c>
       <c r="H149" s="8">
-        <v>209</v>
+        <v>62</v>
       </c>
     </row>
     <row r="150" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7782,7 +7782,7 @@
         <v>14</v>
       </c>
       <c r="H150" s="6">
-        <v>113</v>
+        <v>151</v>
       </c>
     </row>
     <row r="151" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7808,7 +7808,7 @@
         <v>14</v>
       </c>
       <c r="H151" s="8">
-        <v>176</v>
+        <v>199</v>
       </c>
     </row>
     <row r="152" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7834,7 +7834,7 @@
         <v>14</v>
       </c>
       <c r="H152" s="6">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="153" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7860,7 +7860,7 @@
         <v>14</v>
       </c>
       <c r="H153" s="8">
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="154" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7886,7 +7886,7 @@
         <v>14</v>
       </c>
       <c r="H154" s="6">
-        <v>217</v>
+        <v>435</v>
       </c>
     </row>
     <row r="155" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7912,7 +7912,7 @@
         <v>14</v>
       </c>
       <c r="H155" s="8">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="156" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7938,7 +7938,7 @@
         <v>14</v>
       </c>
       <c r="H156" s="6">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="157" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7964,7 +7964,7 @@
         <v>14</v>
       </c>
       <c r="H157" s="8">
-        <v>52</v>
+        <v>74</v>
       </c>
     </row>
     <row r="158" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7990,7 +7990,7 @@
         <v>14</v>
       </c>
       <c r="H158" s="6">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="159" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8016,7 +8016,7 @@
         <v>14</v>
       </c>
       <c r="H159" s="8">
-        <v>125</v>
+        <v>32</v>
       </c>
     </row>
     <row r="160" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8042,7 +8042,7 @@
         <v>14</v>
       </c>
       <c r="H160" s="6">
-        <v>132</v>
+        <v>70</v>
       </c>
     </row>
     <row r="161" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8068,7 +8068,7 @@
         <v>14</v>
       </c>
       <c r="H161" s="8">
-        <v>249</v>
+        <v>365</v>
       </c>
     </row>
     <row r="162" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8094,7 +8094,7 @@
         <v>14</v>
       </c>
       <c r="H162" s="6">
-        <v>109</v>
+        <v>147</v>
       </c>
     </row>
     <row r="163" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8120,7 +8120,7 @@
         <v>14</v>
       </c>
       <c r="H163" s="8">
-        <v>104</v>
+        <v>92</v>
       </c>
     </row>
     <row r="164" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8146,7 +8146,7 @@
         <v>14</v>
       </c>
       <c r="H164" s="6">
-        <v>88</v>
+        <v>131</v>
       </c>
     </row>
     <row r="165" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8172,7 +8172,7 @@
         <v>14</v>
       </c>
       <c r="H165" s="8">
-        <v>205</v>
+        <v>187</v>
       </c>
     </row>
     <row r="166" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8198,7 +8198,7 @@
         <v>14</v>
       </c>
       <c r="H166" s="6">
-        <v>43</v>
+        <v>111</v>
       </c>
     </row>
     <row r="167" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8224,7 +8224,7 @@
         <v>14</v>
       </c>
       <c r="H167" s="8">
-        <v>76</v>
+        <v>166</v>
       </c>
     </row>
     <row r="168" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8250,7 +8250,7 @@
         <v>14</v>
       </c>
       <c r="H168" s="6">
-        <v>59</v>
+        <v>112</v>
       </c>
     </row>
     <row r="169" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8276,7 +8276,7 @@
         <v>14</v>
       </c>
       <c r="H169" s="8">
-        <v>133</v>
+        <v>161</v>
       </c>
     </row>
     <row r="170" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8302,7 +8302,7 @@
         <v>14</v>
       </c>
       <c r="H170" s="6">
-        <v>115</v>
+        <v>150</v>
       </c>
     </row>
     <row r="171" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8328,7 +8328,7 @@
         <v>14</v>
       </c>
       <c r="H171" s="8">
-        <v>148</v>
+        <v>79</v>
       </c>
     </row>
     <row r="172" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>14</v>
       </c>
       <c r="H172" s="6">
-        <v>35</v>
+        <v>144</v>
       </c>
     </row>
     <row r="173" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8380,7 +8380,7 @@
         <v>14</v>
       </c>
       <c r="H173" s="8">
-        <v>114</v>
+        <v>165</v>
       </c>
     </row>
     <row r="174" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8406,7 +8406,7 @@
         <v>14</v>
       </c>
       <c r="H174" s="6">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="175" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8432,7 +8432,7 @@
         <v>14</v>
       </c>
       <c r="H175" s="8">
-        <v>204</v>
+        <v>164</v>
       </c>
     </row>
     <row r="176" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8458,7 +8458,7 @@
         <v>14</v>
       </c>
       <c r="H176" s="6">
-        <v>125</v>
+        <v>145</v>
       </c>
     </row>
     <row r="177" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8484,7 +8484,7 @@
         <v>14</v>
       </c>
       <c r="H177" s="8">
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
     <row r="178" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8510,7 +8510,7 @@
         <v>14</v>
       </c>
       <c r="H178" s="6">
-        <v>49</v>
+        <v>98</v>
       </c>
     </row>
     <row r="179" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8536,7 +8536,7 @@
         <v>14</v>
       </c>
       <c r="H179" s="8">
-        <v>597</v>
+        <v>350</v>
       </c>
     </row>
     <row r="180" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8562,7 +8562,7 @@
         <v>14</v>
       </c>
       <c r="H180" s="6">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="181" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8588,7 +8588,7 @@
         <v>14</v>
       </c>
       <c r="H181" s="8">
-        <v>128</v>
+        <v>185</v>
       </c>
     </row>
     <row r="182" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8614,7 +8614,7 @@
         <v>14</v>
       </c>
       <c r="H182" s="6">
-        <v>70</v>
+        <v>61</v>
       </c>
     </row>
     <row r="183" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8640,7 +8640,7 @@
         <v>14</v>
       </c>
       <c r="H183" s="8">
-        <v>197</v>
+        <v>59</v>
       </c>
     </row>
     <row r="184" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8666,7 +8666,7 @@
         <v>14</v>
       </c>
       <c r="H184" s="6">
-        <v>116</v>
+        <v>201</v>
       </c>
     </row>
     <row r="185" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8692,7 +8692,7 @@
         <v>14</v>
       </c>
       <c r="H185" s="8">
-        <v>131</v>
+        <v>89</v>
       </c>
     </row>
     <row r="186" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8718,7 +8718,7 @@
         <v>14</v>
       </c>
       <c r="H186" s="6">
-        <v>352</v>
+        <v>442</v>
       </c>
     </row>
     <row r="187" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8744,7 +8744,7 @@
         <v>14</v>
       </c>
       <c r="H187" s="8">
-        <v>199</v>
+        <v>101</v>
       </c>
     </row>
     <row r="188" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8770,7 +8770,7 @@
         <v>14</v>
       </c>
       <c r="H188" s="6">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="189" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8796,7 +8796,7 @@
         <v>14</v>
       </c>
       <c r="H189" s="8">
-        <v>146</v>
+        <v>83</v>
       </c>
     </row>
     <row r="190" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8822,7 +8822,7 @@
         <v>14</v>
       </c>
       <c r="H190" s="6">
-        <v>186</v>
+        <v>133</v>
       </c>
     </row>
     <row r="191" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8848,7 +8848,7 @@
         <v>14</v>
       </c>
       <c r="H191" s="8">
-        <v>114</v>
+        <v>155</v>
       </c>
     </row>
     <row r="192" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8874,7 +8874,7 @@
         <v>14</v>
       </c>
       <c r="H192" s="6">
-        <v>183</v>
+        <v>71</v>
       </c>
     </row>
     <row r="193" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8900,7 +8900,7 @@
         <v>14</v>
       </c>
       <c r="H193" s="8">
-        <v>126</v>
+        <v>81</v>
       </c>
     </row>
     <row r="194" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8926,7 +8926,7 @@
         <v>14</v>
       </c>
       <c r="H194" s="6">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="195" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8952,7 +8952,7 @@
         <v>14</v>
       </c>
       <c r="H195" s="8">
-        <v>203</v>
+        <v>53</v>
       </c>
     </row>
     <row r="196" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -8978,7 +8978,7 @@
         <v>14</v>
       </c>
       <c r="H196" s="6">
-        <v>47</v>
+        <v>91</v>
       </c>
     </row>
     <row r="197" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9004,7 +9004,7 @@
         <v>14</v>
       </c>
       <c r="H197" s="8">
-        <v>167</v>
+        <v>103</v>
       </c>
     </row>
     <row r="198" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9030,7 +9030,7 @@
         <v>14</v>
       </c>
       <c r="H198" s="6">
-        <v>35</v>
+        <v>125</v>
       </c>
     </row>
     <row r="199" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9056,7 +9056,7 @@
         <v>14</v>
       </c>
       <c r="H199" s="8">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="200" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9082,7 +9082,7 @@
         <v>14</v>
       </c>
       <c r="H200" s="6">
-        <v>60</v>
+        <v>88</v>
       </c>
     </row>
     <row r="201" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9108,7 +9108,7 @@
         <v>14</v>
       </c>
       <c r="H201" s="8">
-        <v>46</v>
+        <v>137</v>
       </c>
     </row>
     <row r="202" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9134,7 +9134,7 @@
         <v>14</v>
       </c>
       <c r="H202" s="6">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="203" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9160,7 +9160,7 @@
         <v>14</v>
       </c>
       <c r="H203" s="8">
-        <v>78</v>
+        <v>30</v>
       </c>
     </row>
     <row r="204" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9186,7 +9186,7 @@
         <v>14</v>
       </c>
       <c r="H204" s="6">
-        <v>284</v>
+        <v>566</v>
       </c>
     </row>
     <row r="205" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9212,7 +9212,7 @@
         <v>14</v>
       </c>
       <c r="H205" s="8">
-        <v>83</v>
+        <v>93</v>
       </c>
     </row>
     <row r="206" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9238,7 +9238,7 @@
         <v>14</v>
       </c>
       <c r="H206" s="6">
-        <v>127</v>
+        <v>198</v>
       </c>
     </row>
     <row r="207" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9264,7 +9264,7 @@
         <v>14</v>
       </c>
       <c r="H207" s="8">
-        <v>65</v>
+        <v>42</v>
       </c>
     </row>
     <row r="208" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9290,7 +9290,7 @@
         <v>14</v>
       </c>
       <c r="H208" s="6">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="209" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9316,7 +9316,7 @@
         <v>14</v>
       </c>
       <c r="H209" s="8">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="210" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9368,7 +9368,7 @@
         <v>14</v>
       </c>
       <c r="H211" s="8">
-        <v>359</v>
+        <v>376</v>
       </c>
     </row>
     <row r="212" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9394,7 +9394,7 @@
         <v>14</v>
       </c>
       <c r="H212" s="6">
-        <v>204</v>
+        <v>74</v>
       </c>
     </row>
     <row r="213" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9420,7 +9420,7 @@
         <v>14</v>
       </c>
       <c r="H213" s="8">
-        <v>76</v>
+        <v>32</v>
       </c>
     </row>
     <row r="214" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9446,7 +9446,7 @@
         <v>14</v>
       </c>
       <c r="H214" s="6">
-        <v>155</v>
+        <v>131</v>
       </c>
     </row>
     <row r="215" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9472,7 +9472,7 @@
         <v>14</v>
       </c>
       <c r="H215" s="8">
-        <v>176</v>
+        <v>96</v>
       </c>
     </row>
     <row r="216" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9498,7 +9498,7 @@
         <v>14</v>
       </c>
       <c r="H216" s="6">
-        <v>78</v>
+        <v>149</v>
       </c>
     </row>
     <row r="217" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9550,7 +9550,7 @@
         <v>14</v>
       </c>
       <c r="H218" s="6">
-        <v>36</v>
+        <v>101</v>
       </c>
     </row>
     <row r="219" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9576,7 +9576,7 @@
         <v>14</v>
       </c>
       <c r="H219" s="8">
-        <v>176</v>
+        <v>137</v>
       </c>
     </row>
     <row r="220" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9602,7 +9602,7 @@
         <v>14</v>
       </c>
       <c r="H220" s="6">
-        <v>105</v>
+        <v>139</v>
       </c>
     </row>
     <row r="221" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9628,7 +9628,7 @@
         <v>14</v>
       </c>
       <c r="H221" s="8">
-        <v>68</v>
+        <v>122</v>
       </c>
     </row>
     <row r="222" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9654,7 +9654,7 @@
         <v>14</v>
       </c>
       <c r="H222" s="6">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="223" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9680,7 +9680,7 @@
         <v>14</v>
       </c>
       <c r="H223" s="8">
-        <v>75</v>
+        <v>155</v>
       </c>
     </row>
     <row r="224" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9706,7 +9706,7 @@
         <v>14</v>
       </c>
       <c r="H224" s="6">
-        <v>117</v>
+        <v>33</v>
       </c>
     </row>
     <row r="225" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9732,7 +9732,7 @@
         <v>14</v>
       </c>
       <c r="H225" s="8">
-        <v>149</v>
+        <v>163</v>
       </c>
     </row>
     <row r="226" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9758,7 +9758,7 @@
         <v>14</v>
       </c>
       <c r="H226" s="6">
-        <v>133</v>
+        <v>91</v>
       </c>
     </row>
     <row r="227" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9784,7 +9784,7 @@
         <v>14</v>
       </c>
       <c r="H227" s="8">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="228" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9810,7 +9810,7 @@
         <v>14</v>
       </c>
       <c r="H228" s="6">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="229" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9836,7 +9836,7 @@
         <v>14</v>
       </c>
       <c r="H229" s="8">
-        <v>462</v>
+        <v>351</v>
       </c>
     </row>
     <row r="230" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>14</v>
       </c>
       <c r="H230" s="6">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="231" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9888,7 +9888,7 @@
         <v>14</v>
       </c>
       <c r="H231" s="8">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="232" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9914,7 +9914,7 @@
         <v>14</v>
       </c>
       <c r="H232" s="6">
-        <v>18</v>
+        <v>41</v>
       </c>
     </row>
     <row r="233" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9940,7 +9940,7 @@
         <v>14</v>
       </c>
       <c r="H233" s="8">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="234" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9966,7 +9966,7 @@
         <v>14</v>
       </c>
       <c r="H234" s="6">
-        <v>192</v>
+        <v>169</v>
       </c>
     </row>
     <row r="235" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -9992,7 +9992,7 @@
         <v>14</v>
       </c>
       <c r="H235" s="8">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="236" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10018,7 +10018,7 @@
         <v>14</v>
       </c>
       <c r="H236" s="6">
-        <v>304</v>
+        <v>155</v>
       </c>
     </row>
     <row r="237" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10044,7 +10044,7 @@
         <v>14</v>
       </c>
       <c r="H237" s="8">
-        <v>190</v>
+        <v>44</v>
       </c>
     </row>
     <row r="238" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10070,7 +10070,7 @@
         <v>14</v>
       </c>
       <c r="H238" s="6">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="239" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10096,7 +10096,7 @@
         <v>14</v>
       </c>
       <c r="H239" s="8">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="240" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10122,7 +10122,7 @@
         <v>14</v>
       </c>
       <c r="H240" s="6">
-        <v>96</v>
+        <v>55</v>
       </c>
     </row>
     <row r="241" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10148,7 +10148,7 @@
         <v>14</v>
       </c>
       <c r="H241" s="8">
-        <v>189</v>
+        <v>58</v>
       </c>
     </row>
     <row r="242" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10174,7 +10174,7 @@
         <v>14</v>
       </c>
       <c r="H242" s="6">
-        <v>97</v>
+        <v>43</v>
       </c>
     </row>
     <row r="243" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10200,7 +10200,7 @@
         <v>14</v>
       </c>
       <c r="H243" s="8">
-        <v>105</v>
+        <v>78</v>
       </c>
     </row>
     <row r="244" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10226,7 +10226,7 @@
         <v>14</v>
       </c>
       <c r="H244" s="6">
-        <v>79</v>
+        <v>58</v>
       </c>
     </row>
     <row r="245" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10252,7 +10252,7 @@
         <v>14</v>
       </c>
       <c r="H245" s="8">
-        <v>99</v>
+        <v>78</v>
       </c>
     </row>
     <row r="246" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10278,7 +10278,7 @@
         <v>14</v>
       </c>
       <c r="H246" s="6">
-        <v>78</v>
+        <v>37</v>
       </c>
     </row>
     <row r="247" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10304,7 +10304,7 @@
         <v>14</v>
       </c>
       <c r="H247" s="8">
-        <v>144</v>
+        <v>131</v>
       </c>
     </row>
     <row r="248" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10330,7 +10330,7 @@
         <v>14</v>
       </c>
       <c r="H248" s="6">
-        <v>180</v>
+        <v>73</v>
       </c>
     </row>
     <row r="249" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10356,7 +10356,7 @@
         <v>14</v>
       </c>
       <c r="H249" s="8">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="250" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10382,7 +10382,7 @@
         <v>14</v>
       </c>
       <c r="H250" s="6">
-        <v>76</v>
+        <v>36</v>
       </c>
     </row>
     <row r="251" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10408,7 +10408,7 @@
         <v>14</v>
       </c>
       <c r="H251" s="8">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="252" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10434,7 +10434,7 @@
         <v>14</v>
       </c>
       <c r="H252" s="6">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="253" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10460,7 +10460,7 @@
         <v>14</v>
       </c>
       <c r="H253" s="8">
-        <v>90</v>
+        <v>79</v>
       </c>
     </row>
     <row r="254" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10486,7 +10486,7 @@
         <v>14</v>
       </c>
       <c r="H254" s="6">
-        <v>353</v>
+        <v>216</v>
       </c>
     </row>
     <row r="255" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10512,7 +10512,7 @@
         <v>14</v>
       </c>
       <c r="H255" s="8">
-        <v>47</v>
+        <v>22</v>
       </c>
     </row>
     <row r="256" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10538,7 +10538,7 @@
         <v>14</v>
       </c>
       <c r="H256" s="6">
-        <v>109</v>
+        <v>252</v>
       </c>
     </row>
     <row r="257" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10564,7 +10564,7 @@
         <v>14</v>
       </c>
       <c r="H257" s="8">
-        <v>46</v>
+        <v>63</v>
       </c>
     </row>
     <row r="258" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10590,7 +10590,7 @@
         <v>14</v>
       </c>
       <c r="H258" s="6">
-        <v>79</v>
+        <v>93</v>
       </c>
     </row>
     <row r="259" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>14</v>
       </c>
       <c r="H259" s="8">
-        <v>41</v>
+        <v>137</v>
       </c>
     </row>
     <row r="260" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10642,7 +10642,7 @@
         <v>14</v>
       </c>
       <c r="H260" s="6">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="261" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10668,7 +10668,7 @@
         <v>14</v>
       </c>
       <c r="H261" s="8">
-        <v>377</v>
+        <v>122</v>
       </c>
     </row>
     <row r="262" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10694,7 +10694,7 @@
         <v>14</v>
       </c>
       <c r="H262" s="6">
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
     <row r="263" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10720,7 +10720,7 @@
         <v>14</v>
       </c>
       <c r="H263" s="8">
-        <v>137</v>
+        <v>58</v>
       </c>
     </row>
     <row r="264" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10746,7 +10746,7 @@
         <v>14</v>
       </c>
       <c r="H264" s="6">
-        <v>37</v>
+        <v>75</v>
       </c>
     </row>
     <row r="265" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10772,7 +10772,7 @@
         <v>14</v>
       </c>
       <c r="H265" s="8">
-        <v>97</v>
+        <v>168</v>
       </c>
     </row>
     <row r="266" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10798,7 +10798,7 @@
         <v>14</v>
       </c>
       <c r="H266" s="6">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="267" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10824,7 +10824,7 @@
         <v>14</v>
       </c>
       <c r="H267" s="8">
-        <v>30</v>
+        <v>169</v>
       </c>
     </row>
     <row r="268" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10850,7 +10850,7 @@
         <v>14</v>
       </c>
       <c r="H268" s="6">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="269" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10876,7 +10876,7 @@
         <v>14</v>
       </c>
       <c r="H269" s="8">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="270" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10902,7 +10902,7 @@
         <v>14</v>
       </c>
       <c r="H270" s="6">
-        <v>152</v>
+        <v>209</v>
       </c>
     </row>
     <row r="271" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10928,7 +10928,7 @@
         <v>14</v>
       </c>
       <c r="H271" s="8">
-        <v>107</v>
+        <v>38</v>
       </c>
     </row>
     <row r="272" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10954,7 +10954,7 @@
         <v>14</v>
       </c>
       <c r="H272" s="6">
-        <v>163</v>
+        <v>99</v>
       </c>
     </row>
     <row r="273" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10980,7 +10980,7 @@
         <v>14</v>
       </c>
       <c r="H273" s="8">
-        <v>73</v>
+        <v>103</v>
       </c>
     </row>
     <row r="274" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11006,7 +11006,7 @@
         <v>14</v>
       </c>
       <c r="H274" s="6">
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="275" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11032,7 +11032,7 @@
         <v>14</v>
       </c>
       <c r="H275" s="8">
-        <v>52</v>
+        <v>142</v>
       </c>
     </row>
     <row r="276" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11058,7 +11058,7 @@
         <v>14</v>
       </c>
       <c r="H276" s="6">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="277" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11084,7 +11084,7 @@
         <v>14</v>
       </c>
       <c r="H277" s="8">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="278" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11110,7 +11110,7 @@
         <v>14</v>
       </c>
       <c r="H278" s="6">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="279" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11136,7 +11136,7 @@
         <v>14</v>
       </c>
       <c r="H279" s="8">
-        <v>273</v>
+        <v>164</v>
       </c>
     </row>
     <row r="280" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11162,7 +11162,7 @@
         <v>14</v>
       </c>
       <c r="H280" s="6">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="281" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11188,7 +11188,7 @@
         <v>14</v>
       </c>
       <c r="H281" s="8">
-        <v>107</v>
+        <v>227</v>
       </c>
     </row>
     <row r="282" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11214,7 +11214,7 @@
         <v>14</v>
       </c>
       <c r="H282" s="6">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="283" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11240,7 +11240,7 @@
         <v>14</v>
       </c>
       <c r="H283" s="8">
-        <v>136</v>
+        <v>176</v>
       </c>
     </row>
     <row r="284" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11266,7 +11266,7 @@
         <v>14</v>
       </c>
       <c r="H284" s="6">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="285" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11292,7 +11292,7 @@
         <v>14</v>
       </c>
       <c r="H285" s="8">
-        <v>76</v>
+        <v>131</v>
       </c>
     </row>
     <row r="286" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11318,7 +11318,7 @@
         <v>14</v>
       </c>
       <c r="H286" s="6">
-        <v>315</v>
+        <v>320</v>
       </c>
     </row>
     <row r="287" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11344,7 +11344,7 @@
         <v>14</v>
       </c>
       <c r="H287" s="8">
-        <v>96</v>
+        <v>44</v>
       </c>
     </row>
     <row r="288" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11370,7 +11370,7 @@
         <v>14</v>
       </c>
       <c r="H288" s="6">
-        <v>161</v>
+        <v>37</v>
       </c>
     </row>
     <row r="289" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11396,7 +11396,7 @@
         <v>14</v>
       </c>
       <c r="H289" s="8">
-        <v>58</v>
+        <v>178</v>
       </c>
     </row>
     <row r="290" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11422,7 +11422,7 @@
         <v>14</v>
       </c>
       <c r="H290" s="6">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="291" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11448,7 +11448,7 @@
         <v>14</v>
       </c>
       <c r="H291" s="8">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="292" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11474,7 +11474,7 @@
         <v>14</v>
       </c>
       <c r="H292" s="6">
-        <v>170</v>
+        <v>191</v>
       </c>
     </row>
     <row r="293" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11500,7 +11500,7 @@
         <v>14</v>
       </c>
       <c r="H293" s="8">
-        <v>101</v>
+        <v>176</v>
       </c>
     </row>
     <row r="294" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11552,7 +11552,7 @@
         <v>14</v>
       </c>
       <c r="H295" s="8">
-        <v>89</v>
+        <v>199</v>
       </c>
     </row>
     <row r="296" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11578,7 +11578,7 @@
         <v>14</v>
       </c>
       <c r="H296" s="6">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="297" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11604,7 +11604,7 @@
         <v>14</v>
       </c>
       <c r="H297" s="8">
-        <v>203</v>
+        <v>164</v>
       </c>
     </row>
     <row r="298" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11630,7 +11630,7 @@
         <v>14</v>
       </c>
       <c r="H298" s="6">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="299" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11656,7 +11656,7 @@
         <v>14</v>
       </c>
       <c r="H299" s="8">
-        <v>123</v>
+        <v>108</v>
       </c>
     </row>
     <row r="300" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11682,7 +11682,7 @@
         <v>14</v>
       </c>
       <c r="H300" s="6">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
     <row r="301" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11708,7 +11708,7 @@
         <v>14</v>
       </c>
       <c r="H301" s="8">
-        <v>58</v>
+        <v>203</v>
       </c>
     </row>
     <row r="302" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11734,7 +11734,7 @@
         <v>14</v>
       </c>
       <c r="H302" s="6">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="303" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11760,7 +11760,7 @@
         <v>14</v>
       </c>
       <c r="H303" s="8">
-        <v>82</v>
+        <v>71</v>
       </c>
     </row>
     <row r="304" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11786,7 +11786,7 @@
         <v>14</v>
       </c>
       <c r="H304" s="6">
-        <v>506</v>
+        <v>438</v>
       </c>
     </row>
     <row r="305" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11812,7 +11812,7 @@
         <v>14</v>
       </c>
       <c r="H305" s="8">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="306" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11838,7 +11838,7 @@
         <v>14</v>
       </c>
       <c r="H306" s="6">
-        <v>104</v>
+        <v>184</v>
       </c>
     </row>
     <row r="307" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11864,7 +11864,7 @@
         <v>14</v>
       </c>
       <c r="H307" s="8">
-        <v>41</v>
+        <v>74</v>
       </c>
     </row>
     <row r="308" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11890,7 +11890,7 @@
         <v>14</v>
       </c>
       <c r="H308" s="6">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
     <row r="309" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11916,7 +11916,7 @@
         <v>14</v>
       </c>
       <c r="H309" s="8">
-        <v>98</v>
+        <v>198</v>
       </c>
     </row>
     <row r="310" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11942,7 +11942,7 @@
         <v>14</v>
       </c>
       <c r="H310" s="6">
-        <v>52</v>
+        <v>139</v>
       </c>
     </row>
     <row r="311" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11968,7 +11968,7 @@
         <v>14</v>
       </c>
       <c r="H311" s="8">
-        <v>160</v>
+        <v>208</v>
       </c>
     </row>
     <row r="312" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -11994,7 +11994,7 @@
         <v>14</v>
       </c>
       <c r="H312" s="6">
-        <v>142</v>
+        <v>116</v>
       </c>
     </row>
     <row r="313" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12020,7 +12020,7 @@
         <v>14</v>
       </c>
       <c r="H313" s="8">
-        <v>54</v>
+        <v>102</v>
       </c>
     </row>
     <row r="314" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12046,7 +12046,7 @@
         <v>14</v>
       </c>
       <c r="H314" s="6">
-        <v>77</v>
+        <v>128</v>
       </c>
     </row>
     <row r="315" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12072,7 +12072,7 @@
         <v>14</v>
       </c>
       <c r="H315" s="8">
-        <v>137</v>
+        <v>46</v>
       </c>
     </row>
     <row r="316" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12098,7 +12098,7 @@
         <v>14</v>
       </c>
       <c r="H316" s="6">
-        <v>159</v>
+        <v>47</v>
       </c>
     </row>
     <row r="317" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12124,7 +12124,7 @@
         <v>14</v>
       </c>
       <c r="H317" s="8">
-        <v>75</v>
+        <v>45</v>
       </c>
     </row>
     <row r="318" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12150,7 +12150,7 @@
         <v>14</v>
       </c>
       <c r="H318" s="6">
-        <v>144</v>
+        <v>34</v>
       </c>
     </row>
     <row r="319" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12176,7 +12176,7 @@
         <v>14</v>
       </c>
       <c r="H319" s="8">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="320" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12202,7 +12202,7 @@
         <v>14</v>
       </c>
       <c r="H320" s="6">
-        <v>173</v>
+        <v>87</v>
       </c>
     </row>
     <row r="321" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12228,7 +12228,7 @@
         <v>14</v>
       </c>
       <c r="H321" s="8">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="322" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12254,7 +12254,7 @@
         <v>14</v>
       </c>
       <c r="H322" s="6">
-        <v>113</v>
+        <v>143</v>
       </c>
     </row>
     <row r="323" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12280,7 +12280,7 @@
         <v>14</v>
       </c>
       <c r="H323" s="8">
-        <v>49</v>
+        <v>82</v>
       </c>
     </row>
     <row r="324" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12306,7 +12306,7 @@
         <v>14</v>
       </c>
       <c r="H324" s="6">
-        <v>53</v>
+        <v>131</v>
       </c>
     </row>
     <row r="325" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12332,7 +12332,7 @@
         <v>14</v>
       </c>
       <c r="H325" s="8">
-        <v>34</v>
+        <v>66</v>
       </c>
     </row>
     <row r="326" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12358,7 +12358,7 @@
         <v>14</v>
       </c>
       <c r="H326" s="6">
-        <v>107</v>
+        <v>189</v>
       </c>
     </row>
     <row r="327" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12384,7 +12384,7 @@
         <v>14</v>
       </c>
       <c r="H327" s="8">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="328" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12410,7 +12410,7 @@
         <v>14</v>
       </c>
       <c r="H328" s="6">
-        <v>63</v>
+        <v>95</v>
       </c>
     </row>
     <row r="329" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12436,7 +12436,7 @@
         <v>14</v>
       </c>
       <c r="H329" s="8">
-        <v>483</v>
+        <v>471</v>
       </c>
     </row>
     <row r="330" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12462,7 +12462,7 @@
         <v>14</v>
       </c>
       <c r="H330" s="6">
-        <v>32</v>
+        <v>60</v>
       </c>
     </row>
     <row r="331" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12488,7 +12488,7 @@
         <v>14</v>
       </c>
       <c r="H331" s="8">
-        <v>183</v>
+        <v>218</v>
       </c>
     </row>
     <row r="332" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12514,7 +12514,7 @@
         <v>14</v>
       </c>
       <c r="H332" s="6">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="333" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12540,7 +12540,7 @@
         <v>14</v>
       </c>
       <c r="H333" s="8">
-        <v>100</v>
+        <v>183</v>
       </c>
     </row>
     <row r="334" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12566,7 +12566,7 @@
         <v>14</v>
       </c>
       <c r="H334" s="6">
-        <v>201</v>
+        <v>57</v>
       </c>
     </row>
     <row r="335" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12592,7 +12592,7 @@
         <v>14</v>
       </c>
       <c r="H335" s="8">
-        <v>48</v>
+        <v>73</v>
       </c>
     </row>
     <row r="336" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12618,7 +12618,7 @@
         <v>14</v>
       </c>
       <c r="H336" s="6">
-        <v>115</v>
+        <v>432</v>
       </c>
     </row>
     <row r="337" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>14</v>
       </c>
       <c r="H337" s="8">
-        <v>43</v>
+        <v>80</v>
       </c>
     </row>
     <row r="338" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12670,7 +12670,7 @@
         <v>14</v>
       </c>
       <c r="H338" s="6">
-        <v>71</v>
+        <v>139</v>
       </c>
     </row>
     <row r="339" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12696,7 +12696,7 @@
         <v>14</v>
       </c>
       <c r="H339" s="8">
-        <v>192</v>
+        <v>60</v>
       </c>
     </row>
     <row r="340" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12722,7 +12722,7 @@
         <v>14</v>
       </c>
       <c r="H340" s="6">
-        <v>166</v>
+        <v>133</v>
       </c>
     </row>
     <row r="341" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12748,7 +12748,7 @@
         <v>14</v>
       </c>
       <c r="H341" s="8">
-        <v>55</v>
+        <v>98</v>
       </c>
     </row>
     <row r="342" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12774,7 +12774,7 @@
         <v>14</v>
       </c>
       <c r="H342" s="6">
-        <v>103</v>
+        <v>46</v>
       </c>
     </row>
     <row r="343" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12800,7 +12800,7 @@
         <v>14</v>
       </c>
       <c r="H343" s="8">
-        <v>145</v>
+        <v>66</v>
       </c>
     </row>
     <row r="344" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12826,7 +12826,7 @@
         <v>14</v>
       </c>
       <c r="H344" s="6">
-        <v>116</v>
+        <v>204</v>
       </c>
     </row>
     <row r="345" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12852,7 +12852,7 @@
         <v>14</v>
       </c>
       <c r="H345" s="8">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="346" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12878,7 +12878,7 @@
         <v>14</v>
       </c>
       <c r="H346" s="6">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="347" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12904,7 +12904,7 @@
         <v>14</v>
       </c>
       <c r="H347" s="8">
-        <v>122</v>
+        <v>75</v>
       </c>
     </row>
     <row r="348" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12930,7 +12930,7 @@
         <v>14</v>
       </c>
       <c r="H348" s="6">
-        <v>174</v>
+        <v>154</v>
       </c>
     </row>
     <row r="349" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12956,7 +12956,7 @@
         <v>14</v>
       </c>
       <c r="H349" s="8">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="350" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -12982,7 +12982,7 @@
         <v>14</v>
       </c>
       <c r="H350" s="6">
-        <v>138</v>
+        <v>190</v>
       </c>
     </row>
     <row r="351" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -13008,7 +13008,7 @@
         <v>14</v>
       </c>
       <c r="H351" s="8">
-        <v>83</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>